<commit_message>
Update SH03 Business and agent
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/agent/stf/stf_agent_one_valid_row.xlsx
+++ b/src/test/resources/testData/agent/stf/stf_agent_one_valid_row.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karthik.jaladurgam/Desktop/STOS/Test data/Agent/Automation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/karthik.jaladurgam/workspace/securities-transfer-charge-submissions-ui-tests/src/test/resources/testData/agent/stf/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{385CDDB0-DF55-7D4D-8B44-E07272E7F931}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A69BE2-1524-D142-BD1C-161A95E148B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48011,8 +48011,8 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="R3" r:id="rId1" xr:uid="{B3031FE9-BC7B-8D4F-BC36-659B52911989}"/>
-    <hyperlink ref="T3" r:id="rId2" xr:uid="{376533AD-E232-B147-87BF-8EC7E31BF064}"/>
+    <hyperlink ref="R3" r:id="rId1" xr:uid="{1EEF5596-3DCF-114A-852F-810727A2C038}"/>
+    <hyperlink ref="T3" r:id="rId2" xr:uid="{ECF14D4B-F7C6-604A-9F11-5A9083BCDC50}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>